<commit_message>
Fuzzy dup detection, issues-to-file, fix relay leftover handling
- Add fuzzy duplicate detection: club name variants, same-club athlete
  typos, same-license/different-name pairs, and cross-club same-person
  (same name + same DOB).
- Add --issues-full flag and --issues-out PATH to write the full issue
  report to a text file (useful for sharing with the xlsx owner).
- Fix non_race_only_athlete count inflation: dedup by name-only instead
  of (name, license), so the same person with Banquet/hotel rows under
  blank NRANs isn't counted separately from their race rows.
- Fix relay leftover handling: athletes beyond a full squad of 4 now
  go into a second (incomplete) squad instead of being silently dropped.
  Updates the extra_relay_members NOTE wording to match reality.
- Extend test fixture with fuzzy-duplicate scenarios (every category
  fires exactly once); update EXPECTED_ISSUES.md accordingly.

Change-Id: I491ce42058daa67d045d1888f07e442e21e3b4ce
</commit_message>
<xml_diff>
--- a/tests/test_attendees.xlsx
+++ b/tests/test_attendees.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M441"/>
+  <dimension ref="A1:M449"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18907,6 +18907,342 @@
       <c r="H441" t="inlineStr">
         <is>
           <t>OVERAGE1</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>Varianta</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Clubtyperow</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>clubtv1@x.com</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Open F Obstacle</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>1:33.00</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>Beluga Sauvetage</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>01/01/1998</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>CLUBVAR01</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>Variantb</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Clubtyperow</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>clubtv2@x.com</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Open M Obstacle</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>1:28.00</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>Aurora Test  Club</t>
+        </is>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>01/01/1998</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>CLUBVAR02</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>Henri</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Chiu</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>chiu1@x.com</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Open M Remorquage</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>1:34.00</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>Aurora Test Club</t>
+        </is>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>15/05/1999</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t>CHIU_SAME</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>Henri Tsz Hin</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>Chiu</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>chiu2@x.com</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Open M Remorquage</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>1:34.00</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>Aurora Test Club</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>15/05/1999</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>CHIU_SAME</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>Stephen</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>Kennedy</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>k1@x.com</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>Open M Obstacle</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>2:22.00</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>Elite Rescue</t>
+        </is>
+      </c>
+      <c r="G446" t="inlineStr">
+        <is>
+          <t>06/02/1971</t>
+        </is>
+      </c>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t>KENN01</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>Stphen</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Kennedy</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>k2@x.com</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Open M Obstacle</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>2:23.00</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>Elite Rescue</t>
+        </is>
+      </c>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t>06/02/1971</t>
+        </is>
+      </c>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t>KENN02</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>Gabrielle</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Fortin</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>gf1@x.com</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>Open F Obstacle</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>1:40.00</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>Dauphins de l'Est</t>
+        </is>
+      </c>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t>03/03/2000</t>
+        </is>
+      </c>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t>GFORT_A</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>Gabrielle</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Fortin</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>gf2@x.com</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>Open F Obstacle</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>1:41.00</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>Elite Rescue</t>
+        </is>
+      </c>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t>03/03/2000</t>
+        </is>
+      </c>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t>GFORT_B</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix test xlsx: populate relay teammates so squads form correctly
- Corde entries now paired with teammate field
- Relais Mixte entries list all squad members (newline-separated)
- Result: 57 relay squads + 144 positions written (was 0)

Change-Id: Id9d41e81cb888c7b5919994ef403154a039ed80c
</commit_message>
<xml_diff>
--- a/tests/test_attendees.xlsx
+++ b/tests/test_attendees.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Attendees" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Athlètes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Autres" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendees" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Athlètes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Autres" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -694,6 +694,11 @@
           <t>PEDA02</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Pénélope Poirier POPE03</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -778,6 +783,11 @@
           <t>POPE03</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>David Pelletier PEDA02</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1114,6 +1124,11 @@
           <t>BEHE06</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Kevin Cloutier CLKE07</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1324,6 +1339,11 @@
           <t>CLKE07</t>
         </is>
       </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Héloïse Bélanger BEHE06</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1576,6 +1596,11 @@
           <t>BEVA09</t>
         </is>
       </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Quinn Ouellet OUQU12</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2080,6 +2105,11 @@
           <t>OUQU12</t>
         </is>
       </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Valérie Beaulieu BEVA09</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2416,6 +2446,11 @@
           <t>OUBE14</t>
         </is>
       </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Christophe Lapointe LACH17</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3004,6 +3039,11 @@
           <t>LACH17</t>
         </is>
       </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Béatrice Ouellet OUBE14</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3130,6 +3170,11 @@
           <t>GAFR18</t>
         </is>
       </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Chloé Bergeron BECH19</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3256,6 +3301,11 @@
           <t>BECH19</t>
         </is>
       </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Frédérique Gauthier GAFR18</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3508,6 +3558,11 @@
           <t>GABE21</t>
         </is>
       </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>François Fortin FOFR22</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3550,6 +3605,11 @@
           <t>FOFR22</t>
         </is>
       </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Béatrice Gagné GABE21</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3886,6 +3946,11 @@
           <t>LEMA24</t>
         </is>
       </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>François Simard SIFR26</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4222,6 +4287,11 @@
           <t>SIFR26</t>
         </is>
       </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Maude Leclerc LEMA24</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4432,6 +4502,11 @@
           <t>LECH28</t>
         </is>
       </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Pénélope Lemieux LEPE29</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4558,6 +4633,11 @@
           <t>LEPE29</t>
         </is>
       </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Christophe Lemieux LECH28</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5062,6 +5142,11 @@
           <t>FOCH32</t>
         </is>
       </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Juliette Caron CAJU33</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -5314,6 +5399,11 @@
           <t>CAJU33</t>
         </is>
       </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Chloé Fournier FOCH32</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -5734,6 +5824,11 @@
           <t>CLJU36</t>
         </is>
       </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Gabrielle Leblanc LEGA38</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -5944,6 +6039,11 @@
           <t>LEGA38</t>
         </is>
       </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Juliette Cloutier CLJU36</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -6532,6 +6632,11 @@
           <t>CLSO42</t>
         </is>
       </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>François Morin MOFR50</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -7834,6 +7939,11 @@
           <t>MOFR50</t>
         </is>
       </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>Sophie Cloutier CLSO42</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -7876,6 +7986,11 @@
           <t>BOZA51</t>
         </is>
       </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>Rosalie Gagnon GARO52</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -8170,6 +8285,11 @@
           <t>GARO52</t>
         </is>
       </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>Zachary Boucher BOZA51</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -8338,6 +8458,11 @@
           <t>LEFR53</t>
         </is>
       </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>Inès Cloutier CLIN55</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -8590,6 +8715,11 @@
           <t>CLIN55</t>
         </is>
       </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Frédérique Leclerc LEFR53</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -8884,6 +9014,11 @@
           <t>LETA56</t>
         </is>
       </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>Willow Pelletier PEWI57</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -9094,6 +9229,11 @@
           <t>PEWI57</t>
         </is>
       </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>Tania Lévesque LETA56</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -9304,6 +9444,11 @@
           <t>POYA59</t>
         </is>
       </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>Quentin Leblanc LEQU60</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -9514,6 +9659,11 @@
           <t>LEQU60</t>
         </is>
       </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>Yannick Poirier POYA59</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -10060,6 +10210,11 @@
           <t>POWI63</t>
         </is>
       </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>Quentin Gagnon GAQU64</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -10144,6 +10299,11 @@
           <t>GAQU64</t>
         </is>
       </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>Willow Poirier POWI63</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -10774,6 +10934,11 @@
           <t>BOLE69</t>
         </is>
       </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>Ursula Ouellet OUUR70</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -11110,6 +11275,11 @@
           <t>OUUR70</t>
         </is>
       </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>Léa Boucher BOLE69</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -11446,6 +11616,11 @@
           <t>FOPE72</t>
         </is>
       </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>Xavier Lapointe LAXA75</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -11782,6 +11957,11 @@
           <t>LAXA75</t>
         </is>
       </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>Pénélope Fortin FOPE72</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -11824,6 +12004,11 @@
           <t>LETA76</t>
         </is>
       </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>Emma Tremblay TREM80</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -12496,6 +12681,11 @@
           <t>TREM80</t>
         </is>
       </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>Tania Leclerc LETA76</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -12748,6 +12938,11 @@
           <t>GAEM82</t>
         </is>
       </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>Émile Bouchard BOEM83</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -12832,6 +13027,11 @@
           <t>BOEM83</t>
         </is>
       </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>Emma Gagnon GAEM82</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -13042,6 +13242,11 @@
           <t>BESO84</t>
         </is>
       </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>Yannick Paquette PAYA86</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -13336,6 +13541,11 @@
           <t>PAYA86</t>
         </is>
       </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>Sophie Bergeron BESO84</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -13672,6 +13882,11 @@
           <t>MENO89</t>
         </is>
       </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>Nathaniel Girard GINA90</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -13882,6 +14097,11 @@
           <t>GINA90</t>
         </is>
       </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>Noémie Mercier MENO89</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -14218,6 +14438,11 @@
           <t>LEVA93</t>
         </is>
       </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>Noémie Bergeron BENO95</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -14638,6 +14863,11 @@
           <t>BENO95</t>
         </is>
       </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>Valérie Lemieux LEVA93</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -15352,6 +15582,13 @@
           <t>LAHE01</t>
         </is>
       </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>Juliette Roy ROJU27
+Valérie Beaulieu BEVA09
+David Pelletier PEDA02</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -15394,6 +15631,13 @@
           <t>LAHE01</t>
         </is>
       </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>Juliette Roy ROJU27
+Valérie Beaulieu BEVA09
+David Pelletier PEDA02</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -15436,6 +15680,13 @@
           <t>LAHE01</t>
         </is>
       </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>Juliette Roy ROJU27
+Valérie Beaulieu BEVA09
+David Pelletier PEDA02</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -15478,6 +15729,13 @@
           <t>ROJU27</t>
         </is>
       </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>Héloïse Lavoie LAHE01
+Valérie Beaulieu BEVA09
+David Pelletier PEDA02</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -15520,6 +15778,13 @@
           <t>ROJU27</t>
         </is>
       </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>Héloïse Lavoie LAHE01
+Valérie Beaulieu BEVA09
+David Pelletier PEDA02</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -15562,6 +15827,13 @@
           <t>ROJU27</t>
         </is>
       </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>Héloïse Lavoie LAHE01
+Valérie Beaulieu BEVA09
+David Pelletier PEDA02</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -15604,6 +15876,13 @@
           <t>BEVA09</t>
         </is>
       </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>Héloïse Lavoie LAHE01
+Juliette Roy ROJU27
+David Pelletier PEDA02</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -15646,6 +15925,13 @@
           <t>BEVA09</t>
         </is>
       </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>Héloïse Lavoie LAHE01
+Juliette Roy ROJU27
+David Pelletier PEDA02</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -15688,6 +15974,13 @@
           <t>BEVA09</t>
         </is>
       </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>Héloïse Lavoie LAHE01
+Juliette Roy ROJU27
+David Pelletier PEDA02</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -15730,6 +16023,13 @@
           <t>PEDA02</t>
         </is>
       </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>Héloïse Lavoie LAHE01
+Juliette Roy ROJU27
+Valérie Beaulieu BEVA09</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -15772,6 +16072,13 @@
           <t>PEDA02</t>
         </is>
       </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>Héloïse Lavoie LAHE01
+Juliette Roy ROJU27
+Valérie Beaulieu BEVA09</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -15814,6 +16121,13 @@
           <t>PEDA02</t>
         </is>
       </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>Héloïse Lavoie LAHE01
+Juliette Roy ROJU27
+Valérie Beaulieu BEVA09</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -15856,6 +16170,13 @@
           <t>POLE20</t>
         </is>
       </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>Béatrice Gagné GABE21
+Frédérique Gauthier GAFR18
+Héloïse Bélanger BEHE06</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -15898,6 +16219,13 @@
           <t>POLE20</t>
         </is>
       </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>Béatrice Gagné GABE21
+Frédérique Gauthier GAFR18
+Héloïse Bélanger BEHE06</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -15940,6 +16268,13 @@
           <t>POLE20</t>
         </is>
       </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>Béatrice Gagné GABE21
+Frédérique Gauthier GAFR18
+Héloïse Bélanger BEHE06</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -15982,6 +16317,13 @@
           <t>GABE21</t>
         </is>
       </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>Léa Poirier POLE20
+Frédérique Gauthier GAFR18
+Héloïse Bélanger BEHE06</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -16024,6 +16366,13 @@
           <t>GABE21</t>
         </is>
       </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>Léa Poirier POLE20
+Frédérique Gauthier GAFR18
+Héloïse Bélanger BEHE06</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -16066,6 +16415,13 @@
           <t>GABE21</t>
         </is>
       </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>Léa Poirier POLE20
+Frédérique Gauthier GAFR18
+Héloïse Bélanger BEHE06</t>
+        </is>
+      </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -16108,6 +16464,13 @@
           <t>GAFR18</t>
         </is>
       </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>Léa Poirier POLE20
+Béatrice Gagné GABE21
+Héloïse Bélanger BEHE06</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
@@ -16150,6 +16513,13 @@
           <t>GAFR18</t>
         </is>
       </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>Léa Poirier POLE20
+Béatrice Gagné GABE21
+Héloïse Bélanger BEHE06</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -16192,6 +16562,13 @@
           <t>GAFR18</t>
         </is>
       </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>Léa Poirier POLE20
+Béatrice Gagné GABE21
+Héloïse Bélanger BEHE06</t>
+        </is>
+      </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -16234,6 +16611,13 @@
           <t>BEHE06</t>
         </is>
       </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>Léa Poirier POLE20
+Béatrice Gagné GABE21
+Frédérique Gauthier GAFR18</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -16276,6 +16660,13 @@
           <t>BEHE06</t>
         </is>
       </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>Léa Poirier POLE20
+Béatrice Gagné GABE21
+Frédérique Gauthier GAFR18</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -16318,6 +16709,13 @@
           <t>BEHE06</t>
         </is>
       </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>Léa Poirier POLE20
+Béatrice Gagné GABE21
+Frédérique Gauthier GAFR18</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -16360,6 +16758,14 @@
           <t>BOEM35</t>
         </is>
       </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>Chloé Fournier FOCH32
+Hugo Ouellet OUHU47
+Juliette Caron CAJU33
+Héloïse Roy ROHE34</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -16402,6 +16808,14 @@
           <t>BOEM35</t>
         </is>
       </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>Chloé Fournier FOCH32
+Hugo Ouellet OUHU47
+Juliette Caron CAJU33
+Héloïse Roy ROHE34</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -16444,6 +16858,14 @@
           <t>BOEM35</t>
         </is>
       </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>Chloé Fournier FOCH32
+Hugo Ouellet OUHU47
+Juliette Caron CAJU33
+Héloïse Roy ROHE34</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -16486,6 +16908,14 @@
           <t>FOCH32</t>
         </is>
       </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>Émile Boucher BOEM35
+Hugo Ouellet OUHU47
+Juliette Caron CAJU33
+Héloïse Roy ROHE34</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -16528,6 +16958,14 @@
           <t>FOCH32</t>
         </is>
       </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>Émile Boucher BOEM35
+Hugo Ouellet OUHU47
+Juliette Caron CAJU33
+Héloïse Roy ROHE34</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -16570,6 +17008,14 @@
           <t>FOCH32</t>
         </is>
       </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>Émile Boucher BOEM35
+Hugo Ouellet OUHU47
+Juliette Caron CAJU33
+Héloïse Roy ROHE34</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -16612,6 +17058,14 @@
           <t>OUHU47</t>
         </is>
       </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>Émile Boucher BOEM35
+Chloé Fournier FOCH32
+Juliette Caron CAJU33
+Héloïse Roy ROHE34</t>
+        </is>
+      </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
@@ -16654,6 +17108,14 @@
           <t>OUHU47</t>
         </is>
       </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>Émile Boucher BOEM35
+Chloé Fournier FOCH32
+Juliette Caron CAJU33
+Héloïse Roy ROHE34</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -16696,6 +17158,14 @@
           <t>OUHU47</t>
         </is>
       </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>Émile Boucher BOEM35
+Chloé Fournier FOCH32
+Juliette Caron CAJU33
+Héloïse Roy ROHE34</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -16738,6 +17208,14 @@
           <t>CAJU33</t>
         </is>
       </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>Émile Boucher BOEM35
+Chloé Fournier FOCH32
+Hugo Ouellet OUHU47
+Héloïse Roy ROHE34</t>
+        </is>
+      </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -16780,6 +17258,14 @@
           <t>CAJU33</t>
         </is>
       </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>Émile Boucher BOEM35
+Chloé Fournier FOCH32
+Hugo Ouellet OUHU47
+Héloïse Roy ROHE34</t>
+        </is>
+      </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -16822,6 +17308,14 @@
           <t>CAJU33</t>
         </is>
       </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>Émile Boucher BOEM35
+Chloé Fournier FOCH32
+Hugo Ouellet OUHU47
+Héloïse Roy ROHE34</t>
+        </is>
+      </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -16864,6 +17358,14 @@
           <t>ROHE34</t>
         </is>
       </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>Émile Boucher BOEM35
+Chloé Fournier FOCH32
+Hugo Ouellet OUHU47
+Juliette Caron CAJU33</t>
+        </is>
+      </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -16906,6 +17408,14 @@
           <t>ROHE34</t>
         </is>
       </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>Émile Boucher BOEM35
+Chloé Fournier FOCH32
+Hugo Ouellet OUHU47
+Juliette Caron CAJU33</t>
+        </is>
+      </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -16948,6 +17458,14 @@
           <t>ROHE34</t>
         </is>
       </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>Émile Boucher BOEM35
+Chloé Fournier FOCH32
+Hugo Ouellet OUHU47
+Juliette Caron CAJU33</t>
+        </is>
+      </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -16990,6 +17508,11 @@
           <t>FOFR68</t>
         </is>
       </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>Xavier Cloutier CLXA62</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -17032,6 +17555,11 @@
           <t>FOFR68</t>
         </is>
       </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>Xavier Cloutier CLXA62</t>
+        </is>
+      </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
@@ -17074,6 +17602,11 @@
           <t>FOFR68</t>
         </is>
       </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>Xavier Cloutier CLXA62</t>
+        </is>
+      </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -17116,6 +17649,11 @@
           <t>CLXA62</t>
         </is>
       </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>Frédérique Fournier FOFR68</t>
+        </is>
+      </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -17158,6 +17696,11 @@
           <t>CLXA62</t>
         </is>
       </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>Frédérique Fournier FOFR68</t>
+        </is>
+      </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -17200,6 +17743,11 @@
           <t>CLXA62</t>
         </is>
       </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>Frédérique Fournier FOFR68</t>
+        </is>
+      </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -17242,6 +17790,13 @@
           <t>BESO78</t>
         </is>
       </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>Frédérique Boucher BOFR81
+Benoît Simard SIBE79
+Tania Leclerc LETA76</t>
+        </is>
+      </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -17284,6 +17839,13 @@
           <t>BESO78</t>
         </is>
       </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>Frédérique Boucher BOFR81
+Benoît Simard SIBE79
+Tania Leclerc LETA76</t>
+        </is>
+      </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -17326,6 +17888,13 @@
           <t>BESO78</t>
         </is>
       </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>Frédérique Boucher BOFR81
+Benoît Simard SIBE79
+Tania Leclerc LETA76</t>
+        </is>
+      </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -17368,6 +17937,13 @@
           <t>BOFR81</t>
         </is>
       </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>Sophie Beaulieu BESO78
+Benoît Simard SIBE79
+Tania Leclerc LETA76</t>
+        </is>
+      </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -17410,6 +17986,13 @@
           <t>BOFR81</t>
         </is>
       </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>Sophie Beaulieu BESO78
+Benoît Simard SIBE79
+Tania Leclerc LETA76</t>
+        </is>
+      </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -17452,6 +18035,13 @@
           <t>BOFR81</t>
         </is>
       </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>Sophie Beaulieu BESO78
+Benoît Simard SIBE79
+Tania Leclerc LETA76</t>
+        </is>
+      </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -17494,6 +18084,13 @@
           <t>SIBE79</t>
         </is>
       </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>Sophie Beaulieu BESO78
+Frédérique Boucher BOFR81
+Tania Leclerc LETA76</t>
+        </is>
+      </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
@@ -17536,6 +18133,13 @@
           <t>SIBE79</t>
         </is>
       </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>Sophie Beaulieu BESO78
+Frédérique Boucher BOFR81
+Tania Leclerc LETA76</t>
+        </is>
+      </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
@@ -17578,6 +18182,13 @@
           <t>SIBE79</t>
         </is>
       </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>Sophie Beaulieu BESO78
+Frédérique Boucher BOFR81
+Tania Leclerc LETA76</t>
+        </is>
+      </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -17620,6 +18231,13 @@
           <t>LETA76</t>
         </is>
       </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>Sophie Beaulieu BESO78
+Frédérique Boucher BOFR81
+Benoît Simard SIBE79</t>
+        </is>
+      </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
@@ -17662,6 +18280,13 @@
           <t>LETA76</t>
         </is>
       </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>Sophie Beaulieu BESO78
+Frédérique Boucher BOFR81
+Benoît Simard SIBE79</t>
+        </is>
+      </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
@@ -17704,6 +18329,13 @@
           <t>LETA76</t>
         </is>
       </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>Sophie Beaulieu BESO78
+Frédérique Boucher BOFR81
+Benoît Simard SIBE79</t>
+        </is>
+      </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -17746,6 +18378,13 @@
           <t>BENO95</t>
         </is>
       </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>Yannick Tremblay TRYA92
+Sophie Ouellet OUSO91
+Quinn Beaulieu BEQU98</t>
+        </is>
+      </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
@@ -17788,6 +18427,13 @@
           <t>BENO95</t>
         </is>
       </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>Yannick Tremblay TRYA92
+Sophie Ouellet OUSO91
+Quinn Beaulieu BEQU98</t>
+        </is>
+      </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
@@ -17830,6 +18476,13 @@
           <t>BENO95</t>
         </is>
       </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>Yannick Tremblay TRYA92
+Sophie Ouellet OUSO91
+Quinn Beaulieu BEQU98</t>
+        </is>
+      </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
@@ -17872,6 +18525,13 @@
           <t>TRYA92</t>
         </is>
       </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>Noémie Bergeron BENO95
+Sophie Ouellet OUSO91
+Quinn Beaulieu BEQU98</t>
+        </is>
+      </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
@@ -17914,6 +18574,13 @@
           <t>TRYA92</t>
         </is>
       </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>Noémie Bergeron BENO95
+Sophie Ouellet OUSO91
+Quinn Beaulieu BEQU98</t>
+        </is>
+      </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -17956,6 +18623,13 @@
           <t>TRYA92</t>
         </is>
       </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>Noémie Bergeron BENO95
+Sophie Ouellet OUSO91
+Quinn Beaulieu BEQU98</t>
+        </is>
+      </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
@@ -17998,6 +18672,13 @@
           <t>OUSO91</t>
         </is>
       </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>Noémie Bergeron BENO95
+Yannick Tremblay TRYA92
+Quinn Beaulieu BEQU98</t>
+        </is>
+      </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
@@ -18040,6 +18721,13 @@
           <t>OUSO91</t>
         </is>
       </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>Noémie Bergeron BENO95
+Yannick Tremblay TRYA92
+Quinn Beaulieu BEQU98</t>
+        </is>
+      </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
@@ -18082,6 +18770,13 @@
           <t>OUSO91</t>
         </is>
       </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>Noémie Bergeron BENO95
+Yannick Tremblay TRYA92
+Quinn Beaulieu BEQU98</t>
+        </is>
+      </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
@@ -18124,6 +18819,13 @@
           <t>BEQU98</t>
         </is>
       </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>Noémie Bergeron BENO95
+Yannick Tremblay TRYA92
+Sophie Ouellet OUSO91</t>
+        </is>
+      </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
@@ -18166,6 +18868,13 @@
           <t>BEQU98</t>
         </is>
       </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>Noémie Bergeron BENO95
+Yannick Tremblay TRYA92
+Sophie Ouellet OUSO91</t>
+        </is>
+      </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
@@ -18206,6 +18915,13 @@
       <c r="H423" t="inlineStr">
         <is>
           <t>BEQU98</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>Noémie Bergeron BENO95
+Yannick Tremblay TRYA92
+Sophie Ouellet OUSO91</t>
         </is>
       </c>
     </row>

</xml_diff>